<commit_message>
Special case: True negatives
</commit_message>
<xml_diff>
--- a/test-automation/EN301549v4.1.1-web-automation-matrix.en.xlsx
+++ b/test-automation/EN301549v4.1.1-web-automation-matrix.en.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\github\a11y-best-practices\test-automation\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B2516E7A-E2E8-4C0E-8CB3-D2D42A22D362}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{70EABF83-469B-4E6A-8394-767CC75D70B5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-5130" yWindow="-21720" windowWidth="51840" windowHeight="21840" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-98" yWindow="-98" windowWidth="21795" windowHeight="14116" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Foreword" sheetId="1" r:id="rId1"/>
@@ -120,6 +120,40 @@
 </comments>
 </file>
 
+<file path=xl/comments2.xml><?xml version="1.0" encoding="utf-8"?>
+<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr">
+  <authors>
+    <author>Gottfried Zimmermann</author>
+  </authors>
+  <commentList>
+    <comment ref="C5" authorId="0" shapeId="0" xr:uid="{4340225E-0A54-4AFE-B75A-83F4074D0022}">
+      <text>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Segoe UI"/>
+            <charset val="1"/>
+          </rPr>
+          <t>Gottfried Zimmermann:</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Segoe UI"/>
+            <charset val="1"/>
+          </rPr>
+          <t xml:space="preserve">
+True negatives are ignored for the purpose of averaging over multiple instances of criteria applications.</t>
+        </r>
+      </text>
+    </comment>
+  </commentList>
+</comments>
+</file>
+
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
 <sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="699" uniqueCount="282">
   <si>
@@ -963,24 +997,31 @@
     <t>Meaning wrt negatives</t>
   </si>
   <si>
-    <t>True negative</t>
-  </si>
-  <si>
     <t>False positive, with no or irrelevant/false location information</t>
   </si>
   <si>
     <t>This scale is understood as interval scale, i.e. arithmetic means can be computed.</t>
+  </si>
+  <si>
+    <t>(True negatives)</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr9="http://schemas.microsoft.com/office/spreadsheetml/2016/revision9" mc:Ignorable="x14ac x16r2 xr xr9">
-  <fonts count="22" x14ac:knownFonts="1">
+  <fonts count="25" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
       <scheme val="minor"/>
     </font>
     <font>
@@ -1128,6 +1169,19 @@
       <name val="Segoe UI"/>
       <family val="2"/>
     </font>
+    <font>
+      <sz val="9"/>
+      <color indexed="81"/>
+      <name val="Segoe UI"/>
+      <charset val="1"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="9"/>
+      <color indexed="81"/>
+      <name val="Segoe UI"/>
+      <charset val="1"/>
+    </font>
   </fonts>
   <fills count="8">
     <fill>
@@ -1233,148 +1287,149 @@
   </borders>
   <cellStyleXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0"/>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0"/>
-    <xf numFmtId="9" fontId="9" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0"/>
-    <xf numFmtId="0" fontId="18" fillId="7" borderId="0" applyNumberFormat="0" applyBorder="0"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0"/>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0"/>
+    <xf numFmtId="9" fontId="10" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0"/>
+    <xf numFmtId="0" fontId="19" fillId="7" borderId="0" applyNumberFormat="0" applyBorder="0"/>
   </cellStyleXfs>
-  <cellXfs count="62">
+  <cellXfs count="63">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" textRotation="90" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="1"/>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="1"/>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="1" fontId="13" fillId="0" borderId="2" xfId="3" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="1" fontId="14" fillId="0" borderId="2" xfId="3" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" textRotation="90" wrapText="1"/>
     </xf>
-    <xf numFmtId="1" fontId="13" fillId="0" borderId="3" xfId="3" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="1" fontId="14" fillId="0" borderId="3" xfId="3" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" textRotation="90" wrapText="1"/>
     </xf>
-    <xf numFmtId="1" fontId="3" fillId="0" borderId="2" xfId="3" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="1" fontId="4" fillId="0" borderId="2" xfId="3" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" textRotation="90" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="2" applyFont="1"/>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="2"/>
-    <xf numFmtId="0" fontId="13" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="2" applyFont="1"/>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="2"/>
+    <xf numFmtId="0" fontId="14" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="14" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="15" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" xfId="2" applyFont="1"/>
-    <xf numFmtId="0" fontId="13" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="2" applyFont="1"/>
+    <xf numFmtId="0" fontId="14" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="13" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="14" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="13" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="14" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="13" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="14" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="0" xfId="2" applyFont="1"/>
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="0" xfId="2" applyFont="1"/>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="11" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="13" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="14" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="1" fontId="2" fillId="0" borderId="2" xfId="3" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="1" fontId="3" fillId="0" borderId="2" xfId="3" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" textRotation="90" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="5">
     <cellStyle name="Link" xfId="1" builtinId="8"/>
@@ -1747,7 +1802,7 @@
         <v>163</v>
       </c>
     </row>
-    <row r="5" spans="1:1" ht="28.5" x14ac:dyDescent="0.45">
+    <row r="5" spans="1:1" x14ac:dyDescent="0.45">
       <c r="A5" s="2" t="s">
         <v>164</v>
       </c>
@@ -4777,7 +4832,7 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D496424F-F927-4DEE-86F6-CA0EBBA8D988}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D496424F-F927-4DEE-86F6-CA0EBBA8D988}">
   <dimension ref="A1:C15"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
@@ -4816,8 +4871,8 @@
       <c r="A5">
         <v>0</v>
       </c>
-      <c r="C5" s="60" t="s">
-        <v>279</v>
+      <c r="C5" s="62" t="s">
+        <v>281</v>
       </c>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.45">
@@ -4836,7 +4891,7 @@
         <v>-2</v>
       </c>
       <c r="B7" s="60" t="s">
-        <v>280</v>
+        <v>279</v>
       </c>
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.45">
@@ -4846,7 +4901,7 @@
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A9" s="60" t="s">
-        <v>281</v>
+        <v>280</v>
       </c>
     </row>
     <row r="11" spans="1:3" x14ac:dyDescent="0.45">
@@ -4879,6 +4934,7 @@
     <hyperlink ref="A15" r:id="rId1" display="Wikipedia (2026)" xr:uid="{D62AB9EB-D87E-47CE-A8F5-08F7E0C2AB4F}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.78740157499999996" bottom="0.78740157499999996" header="0.3" footer="0.3"/>
+  <legacyDrawing r:id="rId2"/>
 </worksheet>
 </file>
 

</xml_diff>